<commit_message>
sync excel/2026/日前现货_用电侧小时电价.xlsx from private
</commit_message>
<xml_diff>
--- a/excel/2026/日前现货_用电侧小时电价.xlsx
+++ b/excel/2026/日前现货_用电侧小时电价.xlsx
@@ -1194,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z286"/>
+  <dimension ref="A1:Z291"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:26">
@@ -23963,6 +23963,391 @@
         <v>478.5</v>
       </c>
     </row>
+    <row r="287" spans="1:26">
+      <c r="A287" s="2">
+        <v>46310</v>
+      </c>
+      <c r="C287">
+        <v>499</v>
+      </c>
+      <c r="D287">
+        <v>500</v>
+      </c>
+      <c r="E287">
+        <v>480</v>
+      </c>
+      <c r="F287">
+        <v>479</v>
+      </c>
+      <c r="G287">
+        <v>487.3</v>
+      </c>
+      <c r="H287">
+        <v>498.87</v>
+      </c>
+      <c r="I287">
+        <v>494.93</v>
+      </c>
+      <c r="J287">
+        <v>444.88</v>
+      </c>
+      <c r="K287">
+        <v>396.54</v>
+      </c>
+      <c r="L287">
+        <v>346.18</v>
+      </c>
+      <c r="M287">
+        <v>336.86</v>
+      </c>
+      <c r="N287">
+        <v>333.15</v>
+      </c>
+      <c r="O287">
+        <v>314.65</v>
+      </c>
+      <c r="P287">
+        <v>350</v>
+      </c>
+      <c r="Q287">
+        <v>382</v>
+      </c>
+      <c r="R287">
+        <v>401.3</v>
+      </c>
+      <c r="S287">
+        <v>435.97</v>
+      </c>
+      <c r="T287">
+        <v>439</v>
+      </c>
+      <c r="U287">
+        <v>439.5</v>
+      </c>
+      <c r="V287">
+        <v>411.4</v>
+      </c>
+      <c r="W287">
+        <v>401.5</v>
+      </c>
+      <c r="X287">
+        <v>389</v>
+      </c>
+      <c r="Y287">
+        <v>380.5</v>
+      </c>
+      <c r="Z287">
+        <v>385.95</v>
+      </c>
+    </row>
+    <row r="288" spans="1:26">
+      <c r="A288" s="2">
+        <v>46311</v>
+      </c>
+      <c r="C288">
+        <v>380</v>
+      </c>
+      <c r="D288">
+        <v>320.56</v>
+      </c>
+      <c r="E288">
+        <v>311</v>
+      </c>
+      <c r="F288">
+        <v>307</v>
+      </c>
+      <c r="G288">
+        <v>300</v>
+      </c>
+      <c r="H288">
+        <v>293.05</v>
+      </c>
+      <c r="I288">
+        <v>308.77</v>
+      </c>
+      <c r="J288">
+        <v>319.5</v>
+      </c>
+      <c r="K288">
+        <v>350.35</v>
+      </c>
+      <c r="L288">
+        <v>359.5</v>
+      </c>
+      <c r="M288">
+        <v>380</v>
+      </c>
+      <c r="N288">
+        <v>407.5</v>
+      </c>
+      <c r="O288">
+        <v>399.23</v>
+      </c>
+      <c r="P288">
+        <v>425.5</v>
+      </c>
+      <c r="Q288">
+        <v>403.49</v>
+      </c>
+      <c r="R288">
+        <v>379</v>
+      </c>
+      <c r="S288">
+        <v>368.55</v>
+      </c>
+      <c r="T288">
+        <v>350</v>
+      </c>
+      <c r="U288">
+        <v>344.24</v>
+      </c>
+      <c r="V288">
+        <v>332.5</v>
+      </c>
+      <c r="W288">
+        <v>330.5</v>
+      </c>
+      <c r="X288">
+        <v>328.09</v>
+      </c>
+      <c r="Y288">
+        <v>309.5</v>
+      </c>
+      <c r="Z288">
+        <v>220.5</v>
+      </c>
+    </row>
+    <row r="289" spans="1:26">
+      <c r="A289" s="2">
+        <v>46312</v>
+      </c>
+      <c r="C289">
+        <v>329.91</v>
+      </c>
+      <c r="D289">
+        <v>262</v>
+      </c>
+      <c r="E289">
+        <v>193.38</v>
+      </c>
+      <c r="F289">
+        <v>194.5</v>
+      </c>
+      <c r="G289">
+        <v>182.5</v>
+      </c>
+      <c r="H289">
+        <v>264.85</v>
+      </c>
+      <c r="I289">
+        <v>299.8</v>
+      </c>
+      <c r="J289">
+        <v>259.8</v>
+      </c>
+      <c r="K289">
+        <v>199.5</v>
+      </c>
+      <c r="L289">
+        <v>199.5</v>
+      </c>
+      <c r="M289">
+        <v>100</v>
+      </c>
+      <c r="N289">
+        <v>181.96</v>
+      </c>
+      <c r="O289">
+        <v>165.35</v>
+      </c>
+      <c r="P289">
+        <v>200</v>
+      </c>
+      <c r="Q289">
+        <v>300</v>
+      </c>
+      <c r="R289">
+        <v>414</v>
+      </c>
+      <c r="S289">
+        <v>494.03</v>
+      </c>
+      <c r="T289">
+        <v>535.02</v>
+      </c>
+      <c r="U289">
+        <v>529.88</v>
+      </c>
+      <c r="V289">
+        <v>533.21</v>
+      </c>
+      <c r="W289">
+        <v>530</v>
+      </c>
+      <c r="X289">
+        <v>530</v>
+      </c>
+      <c r="Y289">
+        <v>530</v>
+      </c>
+      <c r="Z289">
+        <v>529.75</v>
+      </c>
+    </row>
+    <row r="290" spans="1:26">
+      <c r="A290" s="2">
+        <v>46313</v>
+      </c>
+      <c r="C290">
+        <v>477.5</v>
+      </c>
+      <c r="D290">
+        <v>468.5</v>
+      </c>
+      <c r="E290">
+        <v>459</v>
+      </c>
+      <c r="F290">
+        <v>455</v>
+      </c>
+      <c r="G290">
+        <v>462.5</v>
+      </c>
+      <c r="H290">
+        <v>461.5</v>
+      </c>
+      <c r="I290">
+        <v>457</v>
+      </c>
+      <c r="J290">
+        <v>455.5</v>
+      </c>
+      <c r="K290">
+        <v>449.23</v>
+      </c>
+      <c r="L290">
+        <v>447.81</v>
+      </c>
+      <c r="M290">
+        <v>416.7</v>
+      </c>
+      <c r="N290">
+        <v>430.5</v>
+      </c>
+      <c r="O290">
+        <v>446.57</v>
+      </c>
+      <c r="P290">
+        <v>492.63</v>
+      </c>
+      <c r="Q290">
+        <v>502.2</v>
+      </c>
+      <c r="R290">
+        <v>497</v>
+      </c>
+      <c r="S290">
+        <v>488.34</v>
+      </c>
+      <c r="T290">
+        <v>493.1</v>
+      </c>
+      <c r="U290">
+        <v>484</v>
+      </c>
+      <c r="V290">
+        <v>475</v>
+      </c>
+      <c r="W290">
+        <v>474.5</v>
+      </c>
+      <c r="X290">
+        <v>470</v>
+      </c>
+      <c r="Y290">
+        <v>474</v>
+      </c>
+      <c r="Z290">
+        <v>463.5</v>
+      </c>
+    </row>
+    <row r="291" spans="1:26">
+      <c r="A291" s="2">
+        <v>46314</v>
+      </c>
+      <c r="C291">
+        <v>469</v>
+      </c>
+      <c r="D291">
+        <v>460</v>
+      </c>
+      <c r="E291">
+        <v>454</v>
+      </c>
+      <c r="F291">
+        <v>452.5</v>
+      </c>
+      <c r="G291">
+        <v>460</v>
+      </c>
+      <c r="H291">
+        <v>465</v>
+      </c>
+      <c r="I291">
+        <v>469.5</v>
+      </c>
+      <c r="J291">
+        <v>471.66</v>
+      </c>
+      <c r="K291">
+        <v>511.39</v>
+      </c>
+      <c r="L291">
+        <v>544.87</v>
+      </c>
+      <c r="M291">
+        <v>543.84</v>
+      </c>
+      <c r="N291">
+        <v>533.6</v>
+      </c>
+      <c r="O291">
+        <v>500.47</v>
+      </c>
+      <c r="P291">
+        <v>493.3</v>
+      </c>
+      <c r="Q291">
+        <v>479.8</v>
+      </c>
+      <c r="R291">
+        <v>469.5</v>
+      </c>
+      <c r="S291">
+        <v>470</v>
+      </c>
+      <c r="T291">
+        <v>469.2</v>
+      </c>
+      <c r="U291">
+        <v>447.18</v>
+      </c>
+      <c r="V291">
+        <v>430</v>
+      </c>
+      <c r="W291">
+        <v>418.31</v>
+      </c>
+      <c r="X291">
+        <v>357.03</v>
+      </c>
+      <c r="Y291">
+        <v>299.5</v>
+      </c>
+      <c r="Z291">
+        <v>260.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>